<commit_message>
align UNLB with existing UNGSC Brindisi entity and add backfill migration
The Brindisi base is already in systemchart.entities as 'UNGSC Brindisi'
(its rebranded UN Global Service Centre name) with rows in the prior
2025/26 PKM cycle. Calling it 'UNLB' in the new pipeline would create a
parallel entity and split the historical record.

Rename the entity in both reference files (peacekeeping_mission_budgets.csv
and the supplement peacekeeping_mission_mandates.csv) from 'UNLB' to
'UNGSC Brindisi', regenerate the pipeline output (entity_long now matches
the DB's "United Nations Logistics Base at Brindisi, Italy" exactly), and
add migration 018 to backfill the 4 missing 2026/27 citations into DB.

Migration 018 is idempotent (ON CONFLICT DO NOTHING on both
source_documents and source_document_citations) so re-running is safe.
</commit_message>
<xml_diff>
--- a/data/processed/pkm2026/all_mandates.xlsx
+++ b/data/processed/pkm2026/all_mandates.xlsx
@@ -3219,12 +3219,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>UNLB</t>
+          <t>UNGSC Brindisi</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>United Nations Logistics Base at Brindisi</t>
+          <t>United Nations Logistics Base at Brindisi, Italy</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -3277,12 +3277,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>UNLB</t>
+          <t>UNGSC Brindisi</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>United Nations Logistics Base at Brindisi</t>
+          <t>United Nations Logistics Base at Brindisi, Italy</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -3335,12 +3335,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>UNLB</t>
+          <t>UNGSC Brindisi</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>United Nations Logistics Base at Brindisi</t>
+          <t>United Nations Logistics Base at Brindisi, Italy</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -3393,12 +3393,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>UNLB</t>
+          <t>UNGSC Brindisi</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>United Nations Logistics Base at Brindisi</t>
+          <t>United Nations Logistics Base at Brindisi, Italy</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>

</xml_diff>